<commit_message>
Add the component list for the MLX90640 to the parts list.
</commit_message>
<xml_diff>
--- a/pcb/Component list RejsaRubberTrac board v1.4 (2019-11-19).xlsx
+++ b/pcb/Component list RejsaRubberTrac board v1.4 (2019-11-19).xlsx
@@ -1,29 +1,53 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\- - - - - - -Däckstempsensor - - - - -\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\morly\OneDrive\デスクトップ\タイヤ温度ログ\RejsaRubberTrac\pcb\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2CF0883-7704-456B-A18B-70A58452AAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30795" windowHeight="13260"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="MLX90621" sheetId="2" r:id="rId1"/>
+    <sheet name="MLX90640" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="components" localSheetId="0">Sheet1!$A$2:$F$41</definedName>
+    <definedName name="components" localSheetId="0">'MLX90621'!$A$2:$F$41</definedName>
+    <definedName name="components" localSheetId="1">'MLX90640'!$C$4:$O$26</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
-<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <connection id="1" name="components" type="6" refreshedVersion="5" background="1" saveData="1">
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
+  <connection id="1" xr16:uid="{00000000-0015-0000-FFFF-FFFF00000000}" name="components" type="6" refreshedVersion="5" background="1" saveData="1">
+    <textPr codePage="65001" sourceFile="D:\Desktop\components.txt" decimal="," thousands=" ">
+      <textFields count="4">
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+      </textFields>
+    </textPr>
+  </connection>
+  <connection id="2" xr16:uid="{5C5A1992-D334-4DBA-8F19-C498353385C5}" name="components1" type="6" refreshedVersion="5" background="1" saveData="1">
     <textPr codePage="65001" sourceFile="D:\Desktop\components.txt" decimal="," thousands=" ">
       <textFields count="4">
         <textField/>
@@ -37,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="134">
   <si>
     <t>Power switch</t>
   </si>
@@ -181,9 +205,6 @@
   </si>
   <si>
     <t>Adafruit Bluefruit nRF52 CPU/BLE board</t>
-  </si>
-  <si>
-    <t>MLX90621-ESF-BAB temp sensor</t>
   </si>
   <si>
     <t>Only needed if you want to use a AA size Li-Ion rechargeable battery</t>
@@ -302,7 +323,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -312,7 +333,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -323,7 +344,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -333,7 +354,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
@@ -369,30 +390,314 @@
   <si>
     <t>Published on Github</t>
   </si>
+  <si>
+    <t>１個当たり</t>
+    <rPh sb="1" eb="2">
+      <t>コ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ア</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>４個</t>
+    <rPh sb="1" eb="2">
+      <t>コ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>数量</t>
+    <rPh sb="0" eb="2">
+      <t>スウリョウ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>金額</t>
+    <rPh sb="0" eb="2">
+      <t>キンガク</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>送料</t>
+    <rPh sb="0" eb="2">
+      <t>ソウリョウ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>小計</t>
+    <rPh sb="0" eb="2">
+      <t>ショウケイ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>納期(日)</t>
+    <rPh sb="0" eb="2">
+      <t>ノウキ</t>
+    </rPh>
+    <rPh sb="2" eb="5">
+      <t>ニチ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>Adafruit Bluefruit nRF52 CPU/BLE board 3406</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>MOUSER</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>nRF52832</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>↑</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://www.digikey.jp/ja/products/detail/adafruit-industries-llc/3406/7034992?s=N4IgTCBcDaIIIBMCGAzATgVwJYBcAEAQgDYYCm62%2BAdgEoBiArGHgMwAsADAGwgC6AvkA</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>digikey</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>Adafruit ESP32-S3 FEATHER 8MB/0MB PSRAM 5323</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://www.digikey.jp/ja/products/detail/adafruit-industries-llc/5323/16376065?_gl=1*gunwoh*_up*MQ..*_gs*MQ..&amp;gclid=CjwKCAjwuePGBhBZEiwAIGCVSwsYnQE6LlCYl4kYyWmUhtdfKg6PYKqDMsFwTPONSrv-ZT9YwsNdCBoCihMQAvD_BwE&amp;gclsrc=aw.ds&amp;gbraid=0AAAAADrbLlgNJWyVMa1ywMmr6j4JYsnei</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>4d</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>ESP32-S3</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>1x12 pin header, 2,54 mm</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://www.mouser.se/ProductDetail/200-TSW11205TS</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>feather基板に付属</t>
+    <rPh sb="7" eb="9">
+      <t>キバン</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>フゾク</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://www.mouser.se/ProductDetail/200-TSW10407GD</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>Shunt jumpers</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>FL4+RL3+FR2+RR1＝10</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <r>
+      <t>MLX90640</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>を使うなら</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>D3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>は</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ジャンパーなので不要</t>
+    </r>
+    <rPh sb="13" eb="14">
+      <t>ツカフヨウ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>MLX90640-ESF-BAA temp sensor</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>U2</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://ja.aliexpress.com/item/1005008180135795.html?spm=a2g0o.order_list.order_list_main.16.2f84585aAo1tKC&amp;gatewayAdapt=glo2jpn</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>アリエク</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>2W</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>110 degree、MOUSERは5731円</t>
+    <rPh sb="22" eb="23">
+      <t>エン</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://ja.aliexpress.com/item/1005004176046297.html?spm=a2g0o.order_list.order_list_main.28.2f84585aAo1tKC&amp;gatewayAdapt=glo2jpn</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>上が品切れなら</t>
+    <rPh sb="0" eb="1">
+      <t>ウエ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>シナギ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://ja.aliexpress.com/item/1005006980614596.html?spm=a2g0o.order_list.order_list_main.33.7654585aeu9k2v&amp;gatewayAdapt=glo2jpn</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>LIPO</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://ja.aliexpress.com/item/1005006421563695.html?spm=a2g0o.order_list.order_list_main.5.7654585aeu9k2v&amp;gatewayAdapt=glo2jpn</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>size "503035"　PHコネクタ ※極性が逆なのでコネクタ差し替え</t>
+    <rPh sb="22" eb="24">
+      <t>キョクセイ</t>
+    </rPh>
+    <rPh sb="25" eb="26">
+      <t>ギャク</t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t>サ</t>
+    </rPh>
+    <rPh sb="35" eb="36">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>https://ja.aliexpress.com/item/32814862683.html?spm=a2g0o.order_list.order_list_main.4.5854585aYz0aIG&amp;gatewayAdapt=glo2jpn</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>size "503035"　PHコネクタ</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>基板</t>
+    <rPh sb="0" eb="2">
+      <t>キバン</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>JLCPCB</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>１枚はセンサマウント用に切り抜き</t>
+    <rPh sb="1" eb="2">
+      <t>マイ</t>
+    </rPh>
+    <rPh sb="10" eb="11">
+      <t>ヨウ</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>ヌ</t>
+    </rPh>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>MLX90621-ESF-BAB temp sensor</t>
+    <phoneticPr fontId="21"/>
+  </si>
+  <si>
+    <t>not needed</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="21" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="Calibri Light"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="major"/>
     </font>
@@ -400,7 +705,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -408,7 +713,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -416,35 +721,35 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -452,7 +757,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -460,14 +765,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -475,14 +780,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -490,7 +795,7 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -498,14 +803,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -513,7 +818,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -521,7 +826,7 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -530,12 +835,81 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="6"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="16"/>
+      <color theme="10"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="ＭＳ ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -715,8 +1089,26 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -831,6 +1223,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -877,7 +1293,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -888,13 +1304,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyFill="1" applyAlignment="1">
@@ -903,54 +1316,112 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="22" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="42" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="42" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="42" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="42" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="11" xfId="42" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" xfId="42" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" xfId="42" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="11" xfId="42" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" xfId="42" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
-    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="20% - アクセント 1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - アクセント 2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - アクセント 3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - アクセント 4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - アクセント 5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - アクセント 6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - アクセント 1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - アクセント 2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - アクセント 3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - アクセント 4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - アクセント 5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - アクセント 6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - アクセント 1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - アクセント 2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - アクセント 3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - アクセント 4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - アクセント 5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - アクセント 6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="アクセント 1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="アクセント 2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="アクセント 3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="アクセント 4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="アクセント 5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="アクセント 6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="タイトル" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="チェック セル" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="どちらでもない" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="ハイパーリンク" xfId="42" builtinId="8"/>
+    <cellStyle name="メモ" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="リンク セル" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="悪い" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="計算" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="警告文" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="見出し 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="見出し 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="見出し 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="見出し 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="集計" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="出力" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="説明文" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="入力" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
+    <cellStyle name="良い" xfId="6" builtinId="26" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -966,7 +1437,11 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="components" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="components" connectionId="1" xr16:uid="{00000000-0016-0000-0000-000000000000}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="components" connectionId="2" xr16:uid="{9A6E9AB0-1C9C-43AD-B9C0-6BA7DE85993F}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1231,306 +1706,306 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F66"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="16.5" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="45.85546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="75.28515625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="88" style="6" customWidth="1"/>
-    <col min="6" max="6" width="56.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.140625" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="7.7265625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="45.81640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="12.54296875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="75.26953125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="88" style="5" customWidth="1"/>
+    <col min="6" max="6" width="56.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.1796875" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C1" s="3" t="s">
         <v>44</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>46</v>
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>31</v>
       </c>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>69</v>
+      <c r="D4" s="6" t="s">
+        <v>68</v>
       </c>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>68</v>
+      <c r="D5" s="6" t="s">
+        <v>67</v>
       </c>
       <c r="E5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>72</v>
+      <c r="D6" s="6" t="s">
+        <v>71</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>70</v>
+      <c r="D7" s="6" t="s">
+        <v>69</v>
       </c>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B9" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="5" t="s">
+      <c r="D9" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
-        <v>57</v>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B10" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F10" s="5" t="s">
+      <c r="D10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="91" x14ac:dyDescent="0.2">
       <c r="B11" s="2" t="s">
-        <v>48</v>
+        <v>132</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D12" s="7"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="E11" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D12" s="6"/>
+      <c r="E12" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E14" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B15" s="2" t="s">
         <v>30</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B16" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D16" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B17" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D17" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B20" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="6" t="s">
         <v>39</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B21" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>56</v>
+      <c r="D21" s="6" t="s">
+        <v>55</v>
       </c>
       <c r="E21" s="2"/>
-      <c r="F21" s="5" t="s">
+      <c r="F21" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B22" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D22" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="F22" s="5" t="s">
+      <c r="D22" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="4" t="s">
-        <v>57</v>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B23" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F23" s="5" t="s">
+      <c r="D23" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="4" t="s">
-        <v>57</v>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B24" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F24" s="5" t="s">
+      <c r="D24" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="135" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="117" x14ac:dyDescent="0.2">
       <c r="B28" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D28" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E30" s="2"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E31" s="2"/>
     </row>
-    <row r="32" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="13" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
         <v>27</v>
@@ -1538,14 +2013,14 @@
       <c r="C34" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>73</v>
+      <c r="D34" s="6" t="s">
+        <v>72</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="13" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2" t="s">
         <v>29</v>
@@ -1553,27 +2028,27 @@
       <c r="C35" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>71</v>
+      <c r="D35" s="6" t="s">
+        <v>70</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="13" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
-      <c r="D36" s="7"/>
+      <c r="D36" s="6"/>
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" ht="13" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
-      <c r="B37" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D37" s="7"/>
+      <c r="B37" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37" s="6"/>
       <c r="E37" s="2"/>
     </row>
-    <row r="38" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" ht="13" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2" t="s">
         <v>5</v>
@@ -1581,14 +2056,14 @@
       <c r="C38" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="6" t="s">
         <v>33</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="13" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2" t="s">
         <v>6</v>
@@ -1596,134 +2071,797 @@
       <c r="C39" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="6" t="s">
         <v>32</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="13" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>63</v>
+        <v>50</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="E40" s="2"/>
     </row>
-    <row r="41" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" ht="13" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>64</v>
+        <v>51</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>63</v>
       </c>
       <c r="E41" s="2"/>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="13" x14ac:dyDescent="0.2">
+      <c r="A52" s="2"/>
+    </row>
+    <row r="53" spans="1:2" ht="13" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" ht="15" x14ac:dyDescent="0.25">
-      <c r="A52" s="2"/>
-    </row>
-    <row r="53" spans="1:2" ht="15" x14ac:dyDescent="0.25">
-      <c r="A53" s="2" t="s">
+      <c r="B53" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="13" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="15" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
+      <c r="B54" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
     </row>
-    <row r="58" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
     </row>
-    <row r="59" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
     </row>
-    <row r="60" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
     </row>
-    <row r="61" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
     </row>
-    <row r="62" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
     </row>
-    <row r="63" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
     </row>
-    <row r="64" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" ht="13" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
     </row>
-    <row r="65" spans="1:1" ht="15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" ht="13" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
     </row>
-    <row r="66" spans="1:1" ht="15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" ht="13" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="21"/>
   <hyperlinks>
-    <hyperlink ref="F9" r:id="rId1"/>
-    <hyperlink ref="D28" r:id="rId2" display="https://www.ebay.com/sch/i.html?_nkw=vl53l0x&amp;_sop=15"/>
-    <hyperlink ref="D41" r:id="rId3"/>
-    <hyperlink ref="D3" r:id="rId4"/>
-    <hyperlink ref="D8" r:id="rId5"/>
-    <hyperlink ref="D11" r:id="rId6"/>
-    <hyperlink ref="D9" r:id="rId7"/>
-    <hyperlink ref="D10" r:id="rId8"/>
-    <hyperlink ref="D15" r:id="rId9"/>
-    <hyperlink ref="D16" r:id="rId10"/>
-    <hyperlink ref="D20" r:id="rId11"/>
-    <hyperlink ref="D21" r:id="rId12"/>
-    <hyperlink ref="D22" r:id="rId13"/>
-    <hyperlink ref="D23" r:id="rId14"/>
-    <hyperlink ref="D24" r:id="rId15"/>
-    <hyperlink ref="D38" r:id="rId16"/>
-    <hyperlink ref="D39" r:id="rId17"/>
-    <hyperlink ref="D40" r:id="rId18"/>
-    <hyperlink ref="D32" r:id="rId19"/>
-    <hyperlink ref="F10" r:id="rId20"/>
-    <hyperlink ref="F21" r:id="rId21"/>
-    <hyperlink ref="F22" r:id="rId22"/>
-    <hyperlink ref="F23" r:id="rId23"/>
-    <hyperlink ref="F24" r:id="rId24"/>
-    <hyperlink ref="D5" r:id="rId25"/>
-    <hyperlink ref="D6" r:id="rId26"/>
-    <hyperlink ref="D34" r:id="rId27"/>
+    <hyperlink ref="F9" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D28" r:id="rId2" display="https://www.ebay.com/sch/i.html?_nkw=vl53l0x&amp;_sop=15" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D41" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D3" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="D11" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="D9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="D10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D16" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D20" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="D21" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="D22" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="D23" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="D24" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="D38" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="D39" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="D40" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="D32" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="F10" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="F21" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="F22" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="F23" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="F24" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="D5" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="D6" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="D34" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId28"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F00045E-B09B-45B1-A1DE-6DD874594E49}">
+  <dimension ref="C1:O50"/>
+  <sheetFormatPr defaultColWidth="9.90625" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="9.90625" style="2"/>
+    <col min="3" max="3" width="8.453125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="50" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.7265625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="82.08984375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.36328125" style="2" customWidth="1"/>
+    <col min="8" max="10" width="13.08984375" style="2" customWidth="1"/>
+    <col min="11" max="11" width="23.1796875" style="12" customWidth="1"/>
+    <col min="12" max="13" width="23.1796875" style="13" customWidth="1"/>
+    <col min="14" max="14" width="96" style="5" customWidth="1"/>
+    <col min="15" max="15" width="61.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="28.453125" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.90625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="3:15" ht="23.5" x14ac:dyDescent="0.2">
+      <c r="E1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="M1" s="9"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="3:15" ht="23.5" x14ac:dyDescent="0.2">
+      <c r="K2" s="10">
+        <f>SUM(K4:K29)</f>
+        <v>8385.9500000000007</v>
+      </c>
+      <c r="L2" s="11">
+        <f>K2*4</f>
+        <v>33543.800000000003</v>
+      </c>
+      <c r="M2" s="11"/>
+      <c r="N2" s="2"/>
+    </row>
+    <row r="3" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="N3" s="2"/>
+    </row>
+    <row r="4" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="C4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="N4" s="2"/>
+    </row>
+    <row r="5" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D5" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15">
+        <f>3942*1.1</f>
+        <v>4336.2000000000007</v>
+      </c>
+      <c r="J5" s="15"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D6" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="H6" s="15">
+        <v>1</v>
+      </c>
+      <c r="I6" s="15">
+        <f>3939*1.1</f>
+        <v>4332.9000000000005</v>
+      </c>
+      <c r="J6" s="15"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="2"/>
+    </row>
+    <row r="7" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D7" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="H7" s="15">
+        <v>1</v>
+      </c>
+      <c r="I7" s="15">
+        <f>2697*1.1</f>
+        <v>2966.7000000000003</v>
+      </c>
+      <c r="J7" s="15"/>
+      <c r="K7" s="16">
+        <f>H7*I7+J7</f>
+        <v>2966.7000000000003</v>
+      </c>
+      <c r="L7" s="17"/>
+      <c r="M7" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D8" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="G8" s="20"/>
+      <c r="H8" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="21"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="O8" s="18"/>
+    </row>
+    <row r="9" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D9" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="20"/>
+      <c r="H9" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="O9" s="18"/>
+    </row>
+    <row r="10" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D10" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H10" s="15">
+        <v>1</v>
+      </c>
+      <c r="I10" s="15">
+        <v>49</v>
+      </c>
+      <c r="J10" s="15"/>
+      <c r="K10" s="16">
+        <f>H10*I10+J10</f>
+        <v>49</v>
+      </c>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D11" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H11" s="15">
+        <v>1</v>
+      </c>
+      <c r="I11" s="15">
+        <v>96</v>
+      </c>
+      <c r="J11" s="15"/>
+      <c r="K11" s="16">
+        <f>H11*I11+J11</f>
+        <v>96</v>
+      </c>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D12" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H12" s="15">
+        <v>4</v>
+      </c>
+      <c r="I12" s="15">
+        <f>10/4</f>
+        <v>2.5</v>
+      </c>
+      <c r="J12" s="15"/>
+      <c r="K12" s="16">
+        <f>H12*I12+J12</f>
+        <v>10</v>
+      </c>
+      <c r="L12" s="17"/>
+      <c r="M12" s="17"/>
+      <c r="N12" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="13" spans="3:15" x14ac:dyDescent="0.45">
+      <c r="D13" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="20"/>
+      <c r="H13" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="21"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="O13" s="20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D14" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H14" s="15">
+        <v>1</v>
+      </c>
+      <c r="I14" s="15">
+        <v>47</v>
+      </c>
+      <c r="J14" s="15"/>
+      <c r="K14" s="16">
+        <f>H14*I14+J14</f>
+        <v>47</v>
+      </c>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="O14" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D15" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H15" s="15">
+        <v>1</v>
+      </c>
+      <c r="I15" s="15">
+        <v>3164</v>
+      </c>
+      <c r="J15" s="15">
+        <f>672/4</f>
+        <v>168</v>
+      </c>
+      <c r="K15" s="16">
+        <f>H15*I15+J15</f>
+        <v>3332</v>
+      </c>
+      <c r="L15" s="17"/>
+      <c r="M15" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="N15" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="16" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="D16" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="F16" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="H16" s="24">
+        <v>0</v>
+      </c>
+      <c r="I16" s="24">
+        <v>3108</v>
+      </c>
+      <c r="J16" s="24"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="26"/>
+      <c r="N16" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="O16" s="18"/>
+    </row>
+    <row r="18" spans="3:14" ht="26" x14ac:dyDescent="0.2">
+      <c r="C18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N18" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="D19" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H19" s="15">
+        <v>1</v>
+      </c>
+      <c r="I19" s="15">
+        <v>262</v>
+      </c>
+      <c r="J19" s="15"/>
+      <c r="K19" s="16">
+        <f>H19*I19+J19</f>
+        <v>262</v>
+      </c>
+      <c r="L19" s="17"/>
+      <c r="M19" s="17"/>
+    </row>
+    <row r="23" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="C23" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="D24" s="27" t="s">
+        <v>60</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H24" s="5">
+        <v>1</v>
+      </c>
+      <c r="I24" s="5">
+        <v>204</v>
+      </c>
+      <c r="J24" s="5">
+        <f>522/4</f>
+        <v>130.5</v>
+      </c>
+      <c r="K24" s="16">
+        <f>H24*I24+J24</f>
+        <v>334.5</v>
+      </c>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="2"/>
+    </row>
+    <row r="25" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="C26" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="D27" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="F27" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="H27" s="24">
+        <v>1</v>
+      </c>
+      <c r="I27" s="24">
+        <v>674</v>
+      </c>
+      <c r="J27" s="24">
+        <f>874/4</f>
+        <v>218.5</v>
+      </c>
+      <c r="K27" s="16"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="28" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="F28" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H28" s="15">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2">
+        <v>438</v>
+      </c>
+      <c r="J28" s="2">
+        <f>1063/4</f>
+        <v>265.75</v>
+      </c>
+      <c r="K28" s="16">
+        <f>H28*I28+J28</f>
+        <v>703.75</v>
+      </c>
+      <c r="L28" s="17"/>
+      <c r="M28" s="17"/>
+      <c r="N28" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="29" spans="3:14" x14ac:dyDescent="0.2">
+      <c r="D29" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="H29" s="2">
+        <v>2</v>
+      </c>
+      <c r="I29" s="2">
+        <v>250</v>
+      </c>
+      <c r="J29" s="2">
+        <f>850/10</f>
+        <v>85</v>
+      </c>
+      <c r="K29" s="16">
+        <f>H29*I29+J29</f>
+        <v>585</v>
+      </c>
+      <c r="L29" s="17"/>
+      <c r="M29" s="17"/>
+      <c r="N29" s="5" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="35" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C35" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C37" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C38" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C39" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="40" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C40" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="41" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C41" s="2"/>
+    </row>
+    <row r="42" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C42" s="2"/>
+    </row>
+    <row r="43" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C43" s="2"/>
+    </row>
+    <row r="44" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C44" s="2"/>
+    </row>
+    <row r="45" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C45" s="2"/>
+    </row>
+    <row r="46" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C46" s="2"/>
+    </row>
+    <row r="47" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C47" s="2"/>
+    </row>
+    <row r="48" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C48" s="2"/>
+    </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C49" s="2"/>
+    </row>
+    <row r="50" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C50" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="21"/>
+  <hyperlinks>
+    <hyperlink ref="O13" r:id="rId1" xr:uid="{46531E3D-13FD-49EA-B955-43A4854CA618}"/>
+    <hyperlink ref="F5" r:id="rId2" xr:uid="{E0559816-FD68-4DE0-A628-974EB1B92CA9}"/>
+    <hyperlink ref="F12" r:id="rId3" xr:uid="{DF103016-6594-473C-9756-658BD559E8BD}"/>
+    <hyperlink ref="F13" r:id="rId4" xr:uid="{011A04EF-E0D0-44D2-B8A6-6814FF858054}"/>
+    <hyperlink ref="F14" r:id="rId5" xr:uid="{5ACE081E-AD9B-4845-BC3D-FC4D466B5C41}"/>
+    <hyperlink ref="F19" r:id="rId6" xr:uid="{A2BC91DA-2CA8-47DF-90E5-28D3BE36A7CA}"/>
+    <hyperlink ref="O14" r:id="rId7" xr:uid="{1F3F4B1B-6829-48FA-A0E8-628D91DDF384}"/>
+    <hyperlink ref="F9" r:id="rId8" xr:uid="{9B2D9D4B-3151-47DD-A861-AA81AE22D7C5}"/>
+    <hyperlink ref="F10" r:id="rId9" xr:uid="{7C463031-AFAE-480B-B330-5E085ECE641B}"/>
+    <hyperlink ref="F8" r:id="rId10" xr:uid="{783D1B21-E3D9-42EA-AD04-8CD4A4F9F8D3}"/>
+    <hyperlink ref="F11" r:id="rId11" xr:uid="{9634165B-9C3A-4C7F-863F-CE2F70192617}"/>
+    <hyperlink ref="F15" r:id="rId12" xr:uid="{44E5E0CD-D1A7-4A61-A8DF-482D15B849C5}"/>
+    <hyperlink ref="F16" r:id="rId13" xr:uid="{31CEBC63-21C8-4C69-B00C-33DFA885AE5D}"/>
+    <hyperlink ref="F27" r:id="rId14" xr:uid="{7D563AD7-0CBC-4031-9DAC-534D3FA1C114}"/>
+    <hyperlink ref="F24" r:id="rId15" xr:uid="{27CE3F8B-C399-493C-BF75-BA07FFE9C5FA}"/>
+    <hyperlink ref="F28" r:id="rId16" xr:uid="{8D65190F-F205-43D6-8A79-735D2B0E4EFA}"/>
+    <hyperlink ref="F7" r:id="rId17" display="https://www.digikey.jp/ja/products/detail/adafruit-industries-llc/5323/16376065?_gl=1*gunwoh*_up*MQ..*_gs*MQ..&amp;gclid=CjwKCAjwuePGBhBZEiwAIGCVSwsYnQE6LlCYl4kYyWmUhtdfKg6PYKqDMsFwTPONSrv-ZT9YwsNdCBoCihMQAvD_BwE&amp;gclsrc=aw.ds&amp;gbraid=0AAAAADrbLlgNJWyVMa1ywMmr6j4JYsnei" xr:uid="{0F458D44-DB1C-409F-8A80-E7B67EF7D089}"/>
+    <hyperlink ref="F6" r:id="rId18" xr:uid="{AD46503B-A0FD-4834-B488-C0A233F2063F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId19"/>
+</worksheet>
 </file>
</xml_diff>